<commit_message>
scalebay update 2026-05-22 16:02 (183 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>8500</v>
+        <v>8800</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>10500</v>
+        <v>11500</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>8500</v>
+        <v>9500</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>7000</v>
+        <v>7300</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1600</v>
+        <v>1900</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>2000</v>
+        <v>2300</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -906,7 +906,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>15000</v>
+        <v>15300</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
@@ -1030,7 +1030,7 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>13400</v>
+        <v>14400</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
@@ -1096,7 +1096,7 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>13000</v>
+        <v>14000</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>10000</v>
+        <v>10300</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>3500</v>
+        <v>3800</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
@@ -1290,7 +1290,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>3000</v>
+        <v>3300</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -1356,7 +1356,7 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>3500</v>
+        <v>3800</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
@@ -1422,7 +1422,7 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>3300</v>
+        <v>3600</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>6500</v>
+        <v>6800</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
@@ -1550,7 +1550,7 @@
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>14000</v>
+        <v>14600</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>15000</v>
+        <v>15600</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
@@ -1674,7 +1674,7 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
@@ -1732,7 +1732,7 @@
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="2" t="inlineStr">
@@ -1786,7 +1786,7 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>999</v>
+        <v>1999</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>7200</v>
+        <v>8200</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
@@ -1906,7 +1906,7 @@
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>9000</v>
+        <v>9300</v>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr">
@@ -1964,7 +1964,7 @@
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>13000</v>
+        <v>13300</v>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
@@ -2026,7 +2026,7 @@
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>8000</v>
+        <v>8300</v>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
@@ -2088,7 +2088,7 @@
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>7000</v>
+        <v>7300</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>14500</v>
+        <v>15100</v>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
@@ -2216,7 +2216,7 @@
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>3000</v>
+        <v>3300</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
@@ -2274,7 +2274,7 @@
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>4800</v>
+        <v>5100</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>750</v>
+        <v>1750</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
@@ -2394,7 +2394,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>3900</v>
+        <v>4200</v>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
@@ -2460,7 +2460,7 @@
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>4800</v>
+        <v>5100</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
@@ -2526,7 +2526,7 @@
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>4800</v>
+        <v>5100</v>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
@@ -2592,7 +2592,7 @@
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>5999</v>
+        <v>6299</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
@@ -2658,7 +2658,7 @@
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>4700</v>
+        <v>5000</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
@@ -2724,7 +2724,7 @@
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>4800</v>
+        <v>5100</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
@@ -2790,7 +2790,7 @@
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>5300</v>
+        <v>5600</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
@@ -2856,7 +2856,7 @@
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>5800</v>
+        <v>6100</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
@@ -2922,7 +2922,7 @@
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>2900</v>
+        <v>3200</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
@@ -2988,7 +2988,7 @@
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>7800</v>
+        <v>8100</v>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
@@ -3054,7 +3054,7 @@
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>4300</v>
+        <v>4600</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
@@ -3120,7 +3120,7 @@
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>4800</v>
+        <v>5100</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
@@ -3186,7 +3186,7 @@
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>2900</v>
+        <v>3200</v>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
@@ -3252,7 +3252,7 @@
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>4800</v>
+        <v>5100</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
@@ -3318,7 +3318,7 @@
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>5300</v>
+        <v>5600</v>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
@@ -3384,7 +3384,7 @@
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>4300</v>
+        <v>4600</v>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
@@ -3450,7 +3450,7 @@
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>4800</v>
+        <v>5100</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
@@ -3516,7 +3516,7 @@
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>3000</v>
+        <v>3300</v>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
@@ -3578,7 +3578,7 @@
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>3000</v>
+        <v>3300</v>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
@@ -3640,7 +3640,7 @@
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>12000</v>
+        <v>13000</v>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
@@ -3698,7 +3698,7 @@
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>13000</v>
+        <v>14000</v>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
@@ -3756,7 +3756,7 @@
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>9400</v>
+        <v>10400</v>
       </c>
       <c r="G53" s="2" t="inlineStr"/>
       <c r="H53" s="2" t="inlineStr">
@@ -3810,7 +3810,7 @@
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>42000</v>
+        <v>43000</v>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="F55" s="2" t="n">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
@@ -3926,7 +3926,7 @@
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>15000</v>
+        <v>16000</v>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
@@ -3984,7 +3984,7 @@
         </is>
       </c>
       <c r="F57" s="2" t="n">
-        <v>17000</v>
+        <v>18000</v>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
@@ -4042,7 +4042,7 @@
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>6000</v>
+        <v>7000</v>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
@@ -4100,7 +4100,7 @@
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>15000</v>
+        <v>16000</v>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
@@ -4158,7 +4158,7 @@
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>13000</v>
+        <v>14000</v>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
@@ -4216,7 +4216,7 @@
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>30000</v>
+        <v>31000</v>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
@@ -4274,7 +4274,7 @@
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
@@ -4332,7 +4332,7 @@
         </is>
       </c>
       <c r="F63" s="2" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
@@ -4394,7 +4394,7 @@
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>3900</v>
+        <v>4200</v>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
@@ -4456,7 +4456,7 @@
         </is>
       </c>
       <c r="F65" s="2" t="n">
-        <v>5750</v>
+        <v>6050</v>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
@@ -4564,7 +4564,7 @@
         </is>
       </c>
       <c r="F67" s="2" t="n">
-        <v>7950</v>
+        <v>8250</v>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
@@ -4630,7 +4630,7 @@
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>8000</v>
+        <v>8300</v>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
@@ -4696,7 +4696,7 @@
         </is>
       </c>
       <c r="F69" s="2" t="n">
-        <v>3000</v>
+        <v>3300</v>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
@@ -4758,7 +4758,7 @@
         </is>
       </c>
       <c r="F70" s="2" t="n">
-        <v>5500</v>
+        <v>5800</v>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
@@ -4824,7 +4824,7 @@
         </is>
       </c>
       <c r="F71" s="2" t="n">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
@@ -4890,7 +4890,7 @@
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>1300</v>
+        <v>1600</v>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
@@ -4956,7 +4956,7 @@
         </is>
       </c>
       <c r="F73" s="2" t="n">
-        <v>1500</v>
+        <v>1800</v>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
@@ -5022,7 +5022,7 @@
         </is>
       </c>
       <c r="F74" s="2" t="n">
-        <v>900</v>
+        <v>1200</v>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
@@ -5088,7 +5088,7 @@
         </is>
       </c>
       <c r="F75" s="2" t="n">
-        <v>5000</v>
+        <v>5300</v>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
@@ -5154,7 +5154,7 @@
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>5000</v>
+        <v>5300</v>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="F77" s="2" t="n">
-        <v>1300</v>
+        <v>1600</v>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
@@ -5286,7 +5286,7 @@
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>2300</v>
+        <v>2600</v>
       </c>
       <c r="G78" s="2" t="inlineStr"/>
       <c r="H78" s="2" t="inlineStr">
@@ -5344,7 +5344,7 @@
         </is>
       </c>
       <c r="F79" s="2" t="n">
-        <v>2000</v>
+        <v>2300</v>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
@@ -5410,7 +5410,7 @@
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>1000</v>
+        <v>1300</v>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
@@ -5476,7 +5476,7 @@
         </is>
       </c>
       <c r="F81" s="2" t="n">
-        <v>1500</v>
+        <v>1800</v>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
@@ -5542,7 +5542,7 @@
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>1000</v>
+        <v>1300</v>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
@@ -5608,7 +5608,7 @@
         </is>
       </c>
       <c r="F83" s="2" t="n">
-        <v>2500</v>
+        <v>2800</v>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
@@ -5674,7 +5674,7 @@
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>700</v>
+        <v>1000</v>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
@@ -5740,7 +5740,7 @@
         </is>
       </c>
       <c r="F85" s="2" t="n">
-        <v>2700</v>
+        <v>3000</v>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
@@ -5806,7 +5806,7 @@
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>2500</v>
+        <v>2800</v>
       </c>
       <c r="G86" s="2" t="inlineStr"/>
       <c r="H86" s="2" t="inlineStr">
@@ -5868,7 +5868,7 @@
         </is>
       </c>
       <c r="F87" s="2" t="n">
-        <v>5000</v>
+        <v>5300</v>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
@@ -5934,7 +5934,7 @@
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="G88" s="2" t="inlineStr"/>
       <c r="H88" s="2" t="inlineStr">
@@ -5996,7 +5996,7 @@
         </is>
       </c>
       <c r="F89" s="2" t="n">
-        <v>6800</v>
+        <v>7100</v>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
@@ -6062,7 +6062,7 @@
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>1500</v>
+        <v>1800</v>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
@@ -6128,7 +6128,7 @@
         </is>
       </c>
       <c r="F91" s="2" t="n">
-        <v>1400</v>
+        <v>1700</v>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
@@ -6194,7 +6194,7 @@
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>1000</v>
+        <v>1300</v>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
@@ -6260,7 +6260,7 @@
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>2500</v>
+        <v>2800</v>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
@@ -6322,7 +6322,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>12000</v>
+        <v>13000</v>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
@@ -6380,7 +6380,7 @@
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>3999</v>
+        <v>4999</v>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>15000</v>
+        <v>16000</v>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
@@ -6504,7 +6504,7 @@
         </is>
       </c>
       <c r="F97" s="2" t="n">
-        <v>7000</v>
+        <v>8000</v>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
@@ -6566,7 +6566,7 @@
         </is>
       </c>
       <c r="F98" s="2" t="n">
-        <v>25000</v>
+        <v>26000</v>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
@@ -6628,7 +6628,7 @@
         </is>
       </c>
       <c r="F99" s="2" t="n">
-        <v>8000</v>
+        <v>9000</v>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
@@ -6690,7 +6690,7 @@
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>5000</v>
+        <v>6000</v>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
@@ -6752,7 +6752,7 @@
         </is>
       </c>
       <c r="F101" s="2" t="n">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
@@ -6814,7 +6814,7 @@
         </is>
       </c>
       <c r="F102" s="2" t="n">
-        <v>6000</v>
+        <v>7000</v>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
@@ -6876,7 +6876,7 @@
         </is>
       </c>
       <c r="F103" s="2" t="n">
-        <v>9500</v>
+        <v>10500</v>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
@@ -6938,7 +6938,7 @@
         </is>
       </c>
       <c r="F104" s="2" t="n">
-        <v>5000</v>
+        <v>6000</v>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
@@ -7000,7 +7000,7 @@
         </is>
       </c>
       <c r="F105" s="2" t="n">
-        <v>400</v>
+        <v>1400</v>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
@@ -7062,7 +7062,7 @@
         </is>
       </c>
       <c r="F106" s="2" t="n">
-        <v>10000</v>
+        <v>11000</v>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
@@ -7124,7 +7124,7 @@
         </is>
       </c>
       <c r="F107" s="2" t="n">
-        <v>5000</v>
+        <v>6000</v>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
@@ -7186,7 +7186,7 @@
         </is>
       </c>
       <c r="F108" s="2" t="n">
-        <v>4500</v>
+        <v>5500</v>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
@@ -7248,7 +7248,7 @@
         </is>
       </c>
       <c r="F109" s="2" t="n">
-        <v>4450</v>
+        <v>5450</v>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
@@ -7310,7 +7310,7 @@
         </is>
       </c>
       <c r="F110" s="2" t="n">
-        <v>4200</v>
+        <v>5200</v>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
@@ -7372,7 +7372,7 @@
         </is>
       </c>
       <c r="F111" s="2" t="n">
-        <v>3999</v>
+        <v>4999</v>
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
@@ -7434,7 +7434,7 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
@@ -7492,7 +7492,7 @@
         </is>
       </c>
       <c r="F113" s="2" t="n">
-        <v>3700</v>
+        <v>4700</v>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
@@ -7554,7 +7554,7 @@
         </is>
       </c>
       <c r="F114" s="2" t="n">
-        <v>5000</v>
+        <v>6000</v>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
@@ -7616,7 +7616,7 @@
         </is>
       </c>
       <c r="F115" s="2" t="n">
-        <v>500</v>
+        <v>1500</v>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
@@ -7678,7 +7678,7 @@
         </is>
       </c>
       <c r="F116" s="2" t="n">
-        <v>3700</v>
+        <v>4700</v>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
@@ -7740,7 +7740,7 @@
         </is>
       </c>
       <c r="F117" s="2" t="n">
-        <v>3900</v>
+        <v>4900</v>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
@@ -7802,7 +7802,7 @@
         </is>
       </c>
       <c r="F118" s="2" t="n">
-        <v>9000</v>
+        <v>10000</v>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
@@ -7864,7 +7864,7 @@
         </is>
       </c>
       <c r="F119" s="2" t="n">
-        <v>15000</v>
+        <v>16000</v>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
@@ -7926,7 +7926,7 @@
         </is>
       </c>
       <c r="F120" s="2" t="n">
-        <v>15000</v>
+        <v>16000</v>
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
@@ -7988,7 +7988,7 @@
         </is>
       </c>
       <c r="F121" s="2" t="n">
-        <v>7000</v>
+        <v>8000</v>
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
@@ -8050,7 +8050,7 @@
         </is>
       </c>
       <c r="F122" s="2" t="n">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
@@ -8112,7 +8112,7 @@
         </is>
       </c>
       <c r="F123" s="2" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
@@ -8178,7 +8178,7 @@
         </is>
       </c>
       <c r="F124" s="2" t="n">
-        <v>7500</v>
+        <v>8500</v>
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
@@ -8240,7 +8240,7 @@
         </is>
       </c>
       <c r="F125" s="2" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
@@ -8302,7 +8302,7 @@
         </is>
       </c>
       <c r="F126" s="2" t="n">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
@@ -8364,7 +8364,7 @@
         </is>
       </c>
       <c r="F127" s="2" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
@@ -8426,7 +8426,7 @@
         </is>
       </c>
       <c r="F128" s="2" t="n">
-        <v>7900</v>
+        <v>8900</v>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
@@ -8488,7 +8488,7 @@
         </is>
       </c>
       <c r="F129" s="2" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
@@ -8550,7 +8550,7 @@
         </is>
       </c>
       <c r="F130" s="2" t="n">
-        <v>4200</v>
+        <v>5200</v>
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
@@ -8612,7 +8612,7 @@
         </is>
       </c>
       <c r="F131" s="2" t="n">
-        <v>650</v>
+        <v>1650</v>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
@@ -8674,7 +8674,7 @@
         </is>
       </c>
       <c r="F132" s="2" t="n">
-        <v>2600</v>
+        <v>3600</v>
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
@@ -8736,7 +8736,7 @@
         </is>
       </c>
       <c r="F133" s="2" t="n">
-        <v>500</v>
+        <v>1500</v>
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
@@ -8802,7 +8802,7 @@
         </is>
       </c>
       <c r="F134" s="2" t="n">
-        <v>2700</v>
+        <v>3700</v>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
@@ -8860,7 +8860,7 @@
         </is>
       </c>
       <c r="F135" s="2" t="n">
-        <v>2400</v>
+        <v>3400</v>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
@@ -8922,7 +8922,7 @@
         </is>
       </c>
       <c r="F136" s="2" t="n">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
@@ -8984,7 +8984,7 @@
         </is>
       </c>
       <c r="F137" s="2" t="n">
-        <v>12000</v>
+        <v>13000</v>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
@@ -9046,7 +9046,7 @@
         </is>
       </c>
       <c r="F138" s="2" t="n">
-        <v>2600</v>
+        <v>3600</v>
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
@@ -9108,7 +9108,7 @@
         </is>
       </c>
       <c r="F139" s="2" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
@@ -9174,7 +9174,7 @@
         </is>
       </c>
       <c r="F140" s="2" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
@@ -9236,7 +9236,7 @@
         </is>
       </c>
       <c r="F141" s="2" t="n">
-        <v>6500</v>
+        <v>7500</v>
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
@@ -9298,7 +9298,7 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>550</v>
+        <v>1550</v>
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
@@ -9364,7 +9364,7 @@
         </is>
       </c>
       <c r="F143" s="2" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
@@ -9426,7 +9426,7 @@
         </is>
       </c>
       <c r="F144" s="2" t="n">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="G144" s="2" t="inlineStr"/>
       <c r="H144" s="2" t="inlineStr">
@@ -9484,7 +9484,7 @@
         </is>
       </c>
       <c r="F145" s="2" t="n">
-        <v>470</v>
+        <v>1470</v>
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
@@ -9550,7 +9550,7 @@
         </is>
       </c>
       <c r="F146" s="2" t="n">
-        <v>5000</v>
+        <v>6000</v>
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
@@ -9612,7 +9612,7 @@
         </is>
       </c>
       <c r="F147" s="2" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
@@ -9678,7 +9678,7 @@
         </is>
       </c>
       <c r="F148" s="2" t="n">
-        <v>500</v>
+        <v>1500</v>
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
@@ -9744,7 +9744,7 @@
         </is>
       </c>
       <c r="F149" s="2" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
@@ -9802,7 +9802,7 @@
         </is>
       </c>
       <c r="F150" s="2" t="n">
-        <v>6200</v>
+        <v>7200</v>
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
@@ -9864,7 +9864,7 @@
         </is>
       </c>
       <c r="F151" s="2" t="n">
-        <v>2600</v>
+        <v>3600</v>
       </c>
       <c r="G151" s="2" t="inlineStr"/>
       <c r="H151" s="2" t="inlineStr">
@@ -9922,7 +9922,7 @@
         </is>
       </c>
       <c r="F152" s="2" t="n">
-        <v>2200</v>
+        <v>3200</v>
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
@@ -9984,7 +9984,7 @@
         </is>
       </c>
       <c r="F153" s="2" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
@@ -10046,7 +10046,7 @@
         </is>
       </c>
       <c r="F154" s="2" t="n">
-        <v>10000</v>
+        <v>10600</v>
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
@@ -10108,7 +10108,7 @@
         </is>
       </c>
       <c r="F155" s="2" t="n">
-        <v>9000</v>
+        <v>9600</v>
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
@@ -10170,7 +10170,7 @@
         </is>
       </c>
       <c r="F156" s="2" t="n">
-        <v>26000</v>
+        <v>26600</v>
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
@@ -10232,7 +10232,7 @@
         </is>
       </c>
       <c r="F157" s="2" t="n">
-        <v>7400</v>
+        <v>8000</v>
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
@@ -10294,7 +10294,7 @@
         </is>
       </c>
       <c r="F158" s="2" t="n">
-        <v>12500</v>
+        <v>13100</v>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
@@ -10356,7 +10356,7 @@
         </is>
       </c>
       <c r="F159" s="2" t="n">
-        <v>2700</v>
+        <v>3300</v>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
@@ -10418,7 +10418,7 @@
         </is>
       </c>
       <c r="F160" s="2" t="n">
-        <v>6800</v>
+        <v>7400</v>
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
@@ -10480,7 +10480,7 @@
         </is>
       </c>
       <c r="F161" s="2" t="n">
-        <v>25000</v>
+        <v>25600</v>
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
@@ -10542,7 +10542,7 @@
         </is>
       </c>
       <c r="F162" s="2" t="n">
-        <v>11000</v>
+        <v>11600</v>
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
@@ -10604,7 +10604,7 @@
         </is>
       </c>
       <c r="F163" s="2" t="n">
-        <v>10000</v>
+        <v>11000</v>
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
@@ -10662,7 +10662,7 @@
         </is>
       </c>
       <c r="F164" s="2" t="n">
-        <v>13000</v>
+        <v>14000</v>
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
@@ -10720,7 +10720,7 @@
         </is>
       </c>
       <c r="F165" s="2" t="n">
-        <v>14500</v>
+        <v>15500</v>
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
@@ -10778,7 +10778,7 @@
         </is>
       </c>
       <c r="F166" s="2" t="n">
-        <v>7000</v>
+        <v>8000</v>
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
@@ -10836,7 +10836,7 @@
         </is>
       </c>
       <c r="F167" s="2" t="n">
-        <v>7500</v>
+        <v>8500</v>
       </c>
       <c r="G167" s="2" t="inlineStr">
         <is>
@@ -10894,7 +10894,7 @@
         </is>
       </c>
       <c r="F168" s="2" t="n">
-        <v>7500</v>
+        <v>8500</v>
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
@@ -10948,7 +10948,7 @@
         </is>
       </c>
       <c r="F169" s="2" t="n">
-        <v>9500</v>
+        <v>10500</v>
       </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
@@ -11006,7 +11006,7 @@
         </is>
       </c>
       <c r="F170" s="2" t="n">
-        <v>9500</v>
+        <v>10500</v>
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
@@ -11072,7 +11072,7 @@
         </is>
       </c>
       <c r="F171" s="2" t="n">
-        <v>6500</v>
+        <v>7500</v>
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
@@ -11134,7 +11134,7 @@
         </is>
       </c>
       <c r="F172" s="2" t="n">
-        <v>6000</v>
+        <v>7000</v>
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
@@ -11196,7 +11196,7 @@
         </is>
       </c>
       <c r="F173" s="2" t="n">
-        <v>4500</v>
+        <v>5500</v>
       </c>
       <c r="G173" s="2" t="inlineStr"/>
       <c r="H173" s="2" t="inlineStr">
@@ -11254,7 +11254,7 @@
         </is>
       </c>
       <c r="F174" s="2" t="n">
-        <v>4450</v>
+        <v>5450</v>
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
@@ -11316,7 +11316,7 @@
         </is>
       </c>
       <c r="F175" s="2" t="n">
-        <v>3600</v>
+        <v>4600</v>
       </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
@@ -11378,7 +11378,7 @@
         </is>
       </c>
       <c r="F176" s="2" t="n">
-        <v>10500</v>
+        <v>11500</v>
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
@@ -11444,7 +11444,7 @@
         </is>
       </c>
       <c r="F177" s="2" t="n">
-        <v>4200</v>
+        <v>5200</v>
       </c>
       <c r="G177" s="2" t="inlineStr">
         <is>
@@ -11510,7 +11510,7 @@
         </is>
       </c>
       <c r="F178" s="2" t="n">
-        <v>15500</v>
+        <v>16500</v>
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
@@ -11576,7 +11576,7 @@
         </is>
       </c>
       <c r="F179" s="2" t="n">
-        <v>3100</v>
+        <v>4100</v>
       </c>
       <c r="G179" s="2" t="inlineStr">
         <is>
@@ -11642,7 +11642,7 @@
         </is>
       </c>
       <c r="F180" s="2" t="n">
-        <v>4500</v>
+        <v>5500</v>
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
@@ -11708,7 +11708,7 @@
         </is>
       </c>
       <c r="F181" s="2" t="n">
-        <v>10800</v>
+        <v>11800</v>
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
@@ -11770,7 +11770,7 @@
         </is>
       </c>
       <c r="F182" s="2" t="n">
-        <v>8000</v>
+        <v>9000</v>
       </c>
       <c r="G182" s="2" t="inlineStr"/>
       <c r="H182" s="2" t="inlineStr">
@@ -11832,7 +11832,7 @@
         </is>
       </c>
       <c r="F183" s="2" t="n">
-        <v>3350</v>
+        <v>4350</v>
       </c>
       <c r="G183" s="2" t="inlineStr">
         <is>
@@ -11898,7 +11898,7 @@
         </is>
       </c>
       <c r="F184" s="2" t="n">
-        <v>4600</v>
+        <v>5600</v>
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scalebay update 2026-05-25 18:13 (189 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -6664,7 +6664,7 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Автокран КС-3577 (500А) Start Scale Models (SSM)</t>
+          <t>Автокран КС-3577 (500А) КАЧЕСТВО = ЦЕНА (ВЫБОРКА)</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -6678,7 +6678,7 @@
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>16000</v>
+        <v>13000</v>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update matched_far.xlsx (780 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N779"/>
+  <dimension ref="A1:N781"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -45927,34 +45927,34 @@
         <v>740</v>
       </c>
       <c r="B741" t="n">
-        <v>188469</v>
+        <v>159729</v>
       </c>
       <c r="C741" t="inlineStr">
         <is>
-          <t>SMART ForTwo Cabriolet Rally A451 2014</t>
+          <t>LINCOLN TownCar Limousine 2000</t>
         </is>
       </c>
       <c r="D741" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-10-at-233229-3.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-10-at-233229-6.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-10-at-233229-5.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-10-at-233229-4.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011330-1.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011330-2.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011330-3.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011333-1.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011330.jpg</t>
         </is>
       </c>
       <c r="E741" t="inlineStr">
         <is>
-          <t>699691</t>
+          <t>6993505</t>
         </is>
       </c>
       <c r="F741" t="n">
-        <v>3900</v>
+        <v>7000</v>
       </c>
       <c r="G741" t="inlineStr">
         <is>
-          <t>Mercedes-Benz</t>
+          <t>Lincoln</t>
         </is>
       </c>
       <c r="H741" t="inlineStr">
         <is>
-          <t>Spark</t>
+          <t>Vitesse</t>
         </is>
       </c>
       <c r="I741" t="inlineStr">
@@ -45969,7 +45969,7 @@
       </c>
       <c r="K741" t="inlineStr">
         <is>
-          <t>B66960171</t>
+          <t>36311</t>
         </is>
       </c>
       <c r="L741" t="inlineStr">
@@ -45979,7 +45979,7 @@
       </c>
       <c r="M741" t="inlineStr">
         <is>
-          <t>SMART ForTwo Cabriolet Rally A451 (2014), red</t>
+          <t>LINCOLN TownCar Limousine 2000, black</t>
         </is>
       </c>
       <c r="N741" t="inlineStr">
@@ -45993,30 +45993,34 @@
         <v>741</v>
       </c>
       <c r="B742" t="n">
-        <v>225421</v>
+        <v>188469</v>
       </c>
       <c r="C742" t="inlineStr">
         <is>
-          <t>Mini John Cooper Works WRC #37 (2012)</t>
+          <t>SMART ForTwo Cabriolet Rally A451 2014</t>
         </is>
       </c>
       <c r="D742" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-13-at-022826.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-13-at-022826-2.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-13-at-022826-1.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-10-at-233229-3.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-10-at-233229-6.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-10-at-233229-5.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-10-at-233229-4.jpg</t>
         </is>
       </c>
       <c r="E742" t="inlineStr">
         <is>
-          <t>6999312</t>
+          <t>699691</t>
         </is>
       </c>
       <c r="F742" t="n">
-        <v>5500</v>
-      </c>
-      <c r="G742" t="inlineStr"/>
+        <v>3900</v>
+      </c>
+      <c r="G742" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
       <c r="H742" t="inlineStr">
         <is>
-          <t>Altaya</t>
+          <t>Spark</t>
         </is>
       </c>
       <c r="I742" t="inlineStr">
@@ -46031,7 +46035,7 @@
       </c>
       <c r="K742" t="inlineStr">
         <is>
-          <t>ATR005</t>
+          <t>B66960171</t>
         </is>
       </c>
       <c r="L742" t="inlineStr">
@@ -46041,7 +46045,7 @@
       </c>
       <c r="M742" t="inlineStr">
         <is>
-          <t>Mini John Cooper Works WRC #37 D.Sordo/C.Del Barrio Rally Monte-Carlo 2012</t>
+          <t>SMART ForTwo Cabriolet Rally A451 (2014), red</t>
         </is>
       </c>
       <c r="N742" t="inlineStr">
@@ -46055,34 +46059,30 @@
         <v>742</v>
       </c>
       <c r="B743" t="n">
-        <v>240618</v>
+        <v>225421</v>
       </c>
       <c r="C743" t="inlineStr">
         <is>
-          <t>FORD Escort Mk.I Twin Cam #16  1968</t>
+          <t>Mini John Cooper Works WRC #37 (2012)</t>
         </is>
       </c>
       <c r="D743" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012215-5.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012215-6.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012215-7.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-13-at-022826.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-13-at-022826-2.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-13-at-022826-1.jpg</t>
         </is>
       </c>
       <c r="E743" t="inlineStr">
         <is>
-          <t>7018990</t>
+          <t>6999312</t>
         </is>
       </c>
       <c r="F743" t="n">
-        <v>3400</v>
-      </c>
-      <c r="G743" t="inlineStr">
-        <is>
-          <t>Ford</t>
-        </is>
-      </c>
+        <v>5500</v>
+      </c>
+      <c r="G743" t="inlineStr"/>
       <c r="H743" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>Altaya</t>
         </is>
       </c>
       <c r="I743" t="inlineStr">
@@ -46097,7 +46097,7 @@
       </c>
       <c r="K743" t="inlineStr">
         <is>
-          <t>4672101</t>
+          <t>ATR005</t>
         </is>
       </c>
       <c r="L743" t="inlineStr">
@@ -46107,7 +46107,7 @@
       </c>
       <c r="M743" t="inlineStr">
         <is>
-          <t>FORD Escort Mk.I Twin Cam #16 Frank Gardner "Alan Mann Racing" BTCC Champion 1968</t>
+          <t>Mini John Cooper Works WRC #37 D.Sordo/C.Del Barrio Rally Monte-Carlo 2012</t>
         </is>
       </c>
       <c r="N743" t="inlineStr">
@@ -46121,34 +46121,34 @@
         <v>743</v>
       </c>
       <c r="B744" t="n">
-        <v>327040</v>
+        <v>240618</v>
       </c>
       <c r="C744" t="inlineStr">
         <is>
-          <t>LANCIA Beta Montecarlo Turbo  №51 (1980)</t>
+          <t>FORD Escort Mk.I Twin Cam #16  1968</t>
         </is>
       </c>
       <c r="D744" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221300-15-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221302-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221302-2-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221300-14-(2).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221302-1-(1).jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012215-5.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012215-6.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012215-7.jpg</t>
         </is>
       </c>
       <c r="E744" t="inlineStr">
         <is>
-          <t>7049948</t>
+          <t>7018990</t>
         </is>
       </c>
       <c r="F744" t="n">
-        <v>4800</v>
+        <v>3400</v>
       </c>
       <c r="G744" t="inlineStr">
         <is>
-          <t>Lancia</t>
+          <t>Ford</t>
         </is>
       </c>
       <c r="H744" t="inlineStr">
         <is>
-          <t>Altaya</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="I744" t="inlineStr">
@@ -46161,7 +46161,11 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K744" t="inlineStr"/>
+      <c r="K744" t="inlineStr">
+        <is>
+          <t>4672101</t>
+        </is>
+      </c>
       <c r="L744" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -46169,7 +46173,7 @@
       </c>
       <c r="M744" t="inlineStr">
         <is>
-          <t>LANCIA Beta Montecarlo Turbo №51 DRM (1980)</t>
+          <t>FORD Escort Mk.I Twin Cam #16 Frank Gardner "Alan Mann Racing" BTCC Champion 1968</t>
         </is>
       </c>
       <c r="N744" t="inlineStr">
@@ -46183,34 +46187,34 @@
         <v>744</v>
       </c>
       <c r="B745" t="n">
-        <v>248157</v>
+        <v>327040</v>
       </c>
       <c r="C745" t="inlineStr">
         <is>
-          <t>​JEEP Wrangler 4x4 Winter Edition 2017</t>
+          <t>LANCIA Beta Montecarlo Turbo  №51 (1980)</t>
         </is>
       </c>
       <c r="D745" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000420_233.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000427_317.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000421_634.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000416_969.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000423_192.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221300-15-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221302-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221302-2-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221300-14-(2).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221302-1-(1).jpg</t>
         </is>
       </c>
       <c r="E745" t="inlineStr">
         <is>
-          <t>7183045</t>
+          <t>7049948</t>
         </is>
       </c>
       <c r="F745" t="n">
-        <v>5000</v>
+        <v>4800</v>
       </c>
       <c r="G745" t="inlineStr">
         <is>
-          <t>Jeep</t>
+          <t>Lancia</t>
         </is>
       </c>
       <c r="H745" t="inlineStr">
         <is>
-          <t>Greenlight Collectibles</t>
+          <t>Altaya</t>
         </is>
       </c>
       <c r="I745" t="inlineStr">
@@ -46223,11 +46227,7 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K745" t="inlineStr">
-        <is>
-          <t>86151</t>
-        </is>
-      </c>
+      <c r="K745" t="inlineStr"/>
       <c r="L745" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -46235,7 +46235,7 @@
       </c>
       <c r="M745" t="inlineStr">
         <is>
-          <t>JEEP Wrangler 4x4 Winter Edition 2017 Xtreme Purple</t>
+          <t>LANCIA Beta Montecarlo Turbo №51 DRM (1980)</t>
         </is>
       </c>
       <c r="N745" t="inlineStr">
@@ -46249,34 +46249,34 @@
         <v>745</v>
       </c>
       <c r="B746" t="n">
-        <v>240619</v>
+        <v>248157</v>
       </c>
       <c r="C746" t="inlineStr">
         <is>
-          <t>BMW M3 (E30) #11 1991</t>
+          <t>​JEEP Wrangler 4x4 Winter Edition 2017</t>
         </is>
       </c>
       <c r="D746" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012214-2.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012214-3.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012214-4.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000420_233.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000427_317.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000421_634.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000416_969.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000423_192.jpg</t>
         </is>
       </c>
       <c r="E746" t="inlineStr">
         <is>
-          <t>7220941</t>
+          <t>7183045</t>
         </is>
       </c>
       <c r="F746" t="n">
-        <v>4200</v>
+        <v>5000</v>
       </c>
       <c r="G746" t="inlineStr">
         <is>
-          <t>BMW</t>
+          <t>Jeep</t>
         </is>
       </c>
       <c r="H746" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>Greenlight Collectibles</t>
         </is>
       </c>
       <c r="I746" t="inlineStr">
@@ -46291,7 +46291,7 @@
       </c>
       <c r="K746" t="inlineStr">
         <is>
-          <t>4672102</t>
+          <t>86151</t>
         </is>
       </c>
       <c r="L746" t="inlineStr">
@@ -46301,7 +46301,7 @@
       </c>
       <c r="M746" t="inlineStr">
         <is>
-          <t>BMW M3 (E30) #11 Will Hoy "VL Motorsport" BTCC Champion 1991</t>
+          <t>JEEP Wrangler 4x4 Winter Edition 2017 Xtreme Purple</t>
         </is>
       </c>
       <c r="N746" t="inlineStr">
@@ -46315,34 +46315,34 @@
         <v>746</v>
       </c>
       <c r="B747" t="n">
-        <v>174357</v>
+        <v>240619</v>
       </c>
       <c r="C747" t="inlineStr">
         <is>
-          <t>LAMBORGHINI Gallardo Superleggera</t>
+          <t>BMW M3 (E30) #11 1991</t>
         </is>
       </c>
       <c r="D747" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220208_990.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220142_649.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220124_577.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220420_719.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220438_953.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220333_487.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220316_116.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012214-2.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012214-3.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012214-4.jpg</t>
         </is>
       </c>
       <c r="E747" t="inlineStr">
         <is>
-          <t>7250346</t>
+          <t>7220941</t>
         </is>
       </c>
       <c r="F747" t="n">
-        <v>4400</v>
+        <v>4200</v>
       </c>
       <c r="G747" t="inlineStr">
         <is>
-          <t>Lamborghini</t>
+          <t>BMW</t>
         </is>
       </c>
       <c r="H747" t="inlineStr">
         <is>
-          <t>Autoart</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="I747" t="inlineStr">
@@ -46357,7 +46357,7 @@
       </c>
       <c r="K747" t="inlineStr">
         <is>
-          <t>54615</t>
+          <t>4672102</t>
         </is>
       </c>
       <c r="L747" t="inlineStr">
@@ -46367,7 +46367,7 @@
       </c>
       <c r="M747" t="inlineStr">
         <is>
-          <t>LAMBORGHINI Gallardo Superleggera</t>
+          <t>BMW M3 (E30) #11 Will Hoy "VL Motorsport" BTCC Champion 1991</t>
         </is>
       </c>
       <c r="N747" t="inlineStr">
@@ -46381,34 +46381,34 @@
         <v>747</v>
       </c>
       <c r="B748" t="n">
-        <v>189538</v>
+        <v>174357</v>
       </c>
       <c r="C748" t="inlineStr">
         <is>
-          <t>BMW Z1</t>
+          <t>LAMBORGHINI Gallardo Superleggera</t>
         </is>
       </c>
       <c r="D748" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-4.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-5.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-3.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-7.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-2.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-6-(1).jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220208_990.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220142_649.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220124_577.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220420_719.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220438_953.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220333_487.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220316_116.jpg</t>
         </is>
       </c>
       <c r="E748" t="inlineStr">
         <is>
-          <t>7256165</t>
+          <t>7250346</t>
         </is>
       </c>
       <c r="F748" t="n">
-        <v>5500</v>
+        <v>4400</v>
       </c>
       <c r="G748" t="inlineStr">
         <is>
-          <t>BMW</t>
+          <t>Lamborghini</t>
         </is>
       </c>
       <c r="H748" t="inlineStr">
         <is>
-          <t>Minichamps</t>
+          <t>Autoart</t>
         </is>
       </c>
       <c r="I748" t="inlineStr">
@@ -46423,7 +46423,7 @@
       </c>
       <c r="K748" t="inlineStr">
         <is>
-          <t>400020101</t>
+          <t>54615</t>
         </is>
       </c>
       <c r="L748" t="inlineStr">
@@ -46433,7 +46433,7 @@
       </c>
       <c r="M748" t="inlineStr">
         <is>
-          <t>BMW Z1 Magicviolett хорошая новая модель с подвижными деталями в родном боксе</t>
+          <t>LAMBORGHINI Gallardo Superleggera</t>
         </is>
       </c>
       <c r="N748" t="inlineStr">
@@ -46447,34 +46447,34 @@
         <v>748</v>
       </c>
       <c r="B749" t="n">
-        <v>221592</v>
+        <v>189538</v>
       </c>
       <c r="C749" t="inlineStr">
         <is>
-          <t>LAMBORGHINI LM 002 4х4 1986</t>
+          <t>BMW Z1</t>
         </is>
       </c>
       <c r="D749" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011337-9.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011337-8.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011337-10.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011337-7.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-4.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-5.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-3.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-7.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-2.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-6-(1).jpg</t>
         </is>
       </c>
       <c r="E749" t="inlineStr">
         <is>
-          <t>7315732</t>
+          <t>7256165</t>
         </is>
       </c>
       <c r="F749" t="n">
-        <v>6000</v>
+        <v>5500</v>
       </c>
       <c r="G749" t="inlineStr">
         <is>
-          <t>Lamborghini</t>
+          <t>BMW</t>
         </is>
       </c>
       <c r="H749" t="inlineStr">
         <is>
-          <t>Altaya</t>
+          <t>Minichamps</t>
         </is>
       </c>
       <c r="I749" t="inlineStr">
@@ -46489,7 +46489,7 @@
       </c>
       <c r="K749" t="inlineStr">
         <is>
-          <t>LAM020</t>
+          <t>400020101</t>
         </is>
       </c>
       <c r="L749" t="inlineStr">
@@ -46499,7 +46499,7 @@
       </c>
       <c r="M749" t="inlineStr">
         <is>
-          <t>LAMBORGHINI LM 002 4х4 1986</t>
+          <t>BMW Z1 Magicviolett хорошая новая модель с подвижными деталями в родном боксе</t>
         </is>
       </c>
       <c r="N749" t="inlineStr">
@@ -46513,34 +46513,34 @@
         <v>749</v>
       </c>
       <c r="B750" t="n">
-        <v>366743</v>
+        <v>221592</v>
       </c>
       <c r="C750" t="inlineStr">
         <is>
-          <t>Berliet GBD 4X4 Fourgon-Pompe Tonne Hors Route Camiva</t>
+          <t>LAMBORGHINI LM 002 4х4 1986</t>
         </is>
       </c>
       <c r="D750" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-05-at-223201.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-05-at-223201-1.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-05-at-223202.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011337-9.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011337-8.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011337-10.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011337-7.jpg</t>
         </is>
       </c>
       <c r="E750" t="inlineStr">
         <is>
-          <t>7417773</t>
+          <t>7315732</t>
         </is>
       </c>
       <c r="F750" t="n">
-        <v>3900</v>
+        <v>6000</v>
       </c>
       <c r="G750" t="inlineStr">
         <is>
-          <t>Berliet</t>
+          <t>Lamborghini</t>
         </is>
       </c>
       <c r="H750" t="inlineStr">
         <is>
-          <t>Hachette</t>
+          <t>Altaya</t>
         </is>
       </c>
       <c r="I750" t="inlineStr">
@@ -46555,7 +46555,7 @@
       </c>
       <c r="K750" t="inlineStr">
         <is>
-          <t>FC059</t>
+          <t>LAM020</t>
         </is>
       </c>
       <c r="L750" t="inlineStr">
@@ -46565,7 +46565,7 @@
       </c>
       <c r="M750" t="inlineStr">
         <is>
-          <t>Berliet GBD 4X4 Fourgon-Pompe Tonne Hors Route Camiva</t>
+          <t>LAMBORGHINI LM 002 4х4 1986</t>
         </is>
       </c>
       <c r="N750" t="inlineStr">
@@ -46579,30 +46579,34 @@
         <v>750</v>
       </c>
       <c r="B751" t="n">
-        <v>223706</v>
+        <v>366743</v>
       </c>
       <c r="C751" t="inlineStr">
         <is>
-          <t>Автоцистерна АЦ-30 (205)</t>
+          <t>Berliet GBD 4X4 Fourgon-Pompe Tonne Hors Route Camiva</t>
         </is>
       </c>
       <c r="D751" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220608_187-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220451_903-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220507_925-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220517_630-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220505_167-(1).jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-05-at-223201.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-05-at-223201-1.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-05-at-223202.jpg</t>
         </is>
       </c>
       <c r="E751" t="inlineStr">
         <is>
-          <t>7453420</t>
+          <t>7417773</t>
         </is>
       </c>
       <c r="F751" t="n">
-        <v>2200</v>
-      </c>
-      <c r="G751" t="inlineStr"/>
+        <v>3900</v>
+      </c>
+      <c r="G751" t="inlineStr">
+        <is>
+          <t>Berliet</t>
+        </is>
+      </c>
       <c r="H751" t="inlineStr">
         <is>
-          <t>Автолегенды СССР журнал от DeAgostini</t>
+          <t>Hachette</t>
         </is>
       </c>
       <c r="I751" t="inlineStr">
@@ -46615,7 +46619,11 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K751" t="inlineStr"/>
+      <c r="K751" t="inlineStr">
+        <is>
+          <t>FC059</t>
+        </is>
+      </c>
       <c r="L751" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -46623,7 +46631,7 @@
       </c>
       <c r="M751" t="inlineStr">
         <is>
-          <t>Автоцистерна АЦ-30 (205)</t>
+          <t>Berliet GBD 4X4 Fourgon-Pompe Tonne Hors Route Camiva</t>
         </is>
       </c>
       <c r="N751" t="inlineStr">
@@ -46637,30 +46645,30 @@
         <v>751</v>
       </c>
       <c r="B752" t="n">
-        <v>186677</v>
+        <v>223706</v>
       </c>
       <c r="C752" t="inlineStr">
         <is>
-          <t>Multiple Gun Motor Carriage M16</t>
+          <t>Автоцистерна АЦ-30 (205)</t>
         </is>
       </c>
       <c r="D752" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230222.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230223.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230223-1.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220608_187-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220451_903-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220507_925-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220517_630-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220505_167-(1).jpg</t>
         </is>
       </c>
       <c r="E752" t="inlineStr">
         <is>
-          <t>7487066</t>
+          <t>7453420</t>
         </is>
       </c>
       <c r="F752" t="n">
-        <v>3850</v>
+        <v>2200</v>
       </c>
       <c r="G752" t="inlineStr"/>
       <c r="H752" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>Автолегенды СССР журнал от DeAgostini</t>
         </is>
       </c>
       <c r="I752" t="inlineStr">
@@ -46673,11 +46681,7 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K752" t="inlineStr">
-        <is>
-          <t>6690003</t>
-        </is>
-      </c>
+      <c r="K752" t="inlineStr"/>
       <c r="L752" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -46685,7 +46689,7 @@
       </c>
       <c r="M752" t="inlineStr">
         <is>
-          <t>Multiple Gun Motor Carriage M16, military green</t>
+          <t>Автоцистерна АЦ-30 (205)</t>
         </is>
       </c>
       <c r="N752" t="inlineStr">
@@ -46699,34 +46703,30 @@
         <v>752</v>
       </c>
       <c r="B753" t="n">
-        <v>221606</v>
+        <v>186677</v>
       </c>
       <c r="C753" t="inlineStr">
         <is>
-          <t>VOLKSWAGEN Golf I GTI 1976 White</t>
+          <t>Multiple Gun Motor Carriage M16</t>
         </is>
       </c>
       <c r="D753" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012216-16.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012216-17.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012216-18.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230222.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230223.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230223-1.jpg</t>
         </is>
       </c>
       <c r="E753" t="inlineStr">
         <is>
-          <t>7508306</t>
+          <t>7487066</t>
         </is>
       </c>
       <c r="F753" t="n">
-        <v>3800</v>
-      </c>
-      <c r="G753" t="inlineStr">
-        <is>
-          <t>Volkswagen</t>
-        </is>
-      </c>
+        <v>3850</v>
+      </c>
+      <c r="G753" t="inlineStr"/>
       <c r="H753" t="inlineStr">
         <is>
-          <t>Altaya</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="I753" t="inlineStr">
@@ -46741,7 +46741,7 @@
       </c>
       <c r="K753" t="inlineStr">
         <is>
-          <t>TA003</t>
+          <t>6690003</t>
         </is>
       </c>
       <c r="L753" t="inlineStr">
@@ -46751,7 +46751,7 @@
       </c>
       <c r="M753" t="inlineStr">
         <is>
-          <t>VOLKSWAGEN Golf I GTI 1976 White</t>
+          <t>Multiple Gun Motor Carriage M16, military green</t>
         </is>
       </c>
       <c r="N753" t="inlineStr">
@@ -46765,29 +46765,29 @@
         <v>753</v>
       </c>
       <c r="B754" t="n">
-        <v>327718</v>
+        <v>221606</v>
       </c>
       <c r="C754" t="inlineStr">
         <is>
-          <t>Mercedes-Benz 300SLR #722</t>
+          <t>VOLKSWAGEN Golf I GTI 1976 White</t>
         </is>
       </c>
       <c r="D754" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-28.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-29.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-30.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-31.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-27.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012216-16.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012216-17.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012216-18.jpg</t>
         </is>
       </c>
       <c r="E754" t="inlineStr">
         <is>
-          <t>7616575</t>
+          <t>7508306</t>
         </is>
       </c>
       <c r="F754" t="n">
-        <v>4000</v>
+        <v>3800</v>
       </c>
       <c r="G754" t="inlineStr">
         <is>
-          <t>Mercedes-Benz</t>
+          <t>Volkswagen</t>
         </is>
       </c>
       <c r="H754" t="inlineStr">
@@ -46805,7 +46805,11 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K754" t="inlineStr"/>
+      <c r="K754" t="inlineStr">
+        <is>
+          <t>TA003</t>
+        </is>
+      </c>
       <c r="L754" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -46813,7 +46817,7 @@
       </c>
       <c r="M754" t="inlineStr">
         <is>
-          <t>Mercedes-Benz 300SLR #722 победитель Mille Miglia 1955 Stilring Moss/Denis Jenkinson (средняя скорость 160км/ч)</t>
+          <t>VOLKSWAGEN Golf I GTI 1976 White</t>
         </is>
       </c>
       <c r="N754" t="inlineStr">
@@ -46827,25 +46831,25 @@
         <v>754</v>
       </c>
       <c r="B755" t="n">
-        <v>173083</v>
+        <v>327718</v>
       </c>
       <c r="C755" t="inlineStr">
         <is>
-          <t>MERCEDES-BENZ 300 SLR Racing Sports Car 1955</t>
+          <t>Mercedes-Benz 300SLR #722</t>
         </is>
       </c>
       <c r="D755" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011339-18.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011339-19.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011339-20.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011339-21.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011339-17.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-28.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-29.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-30.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-31.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-27.jpg</t>
         </is>
       </c>
       <c r="E755" t="inlineStr">
         <is>
-          <t>7710208</t>
+          <t>7616575</t>
         </is>
       </c>
       <c r="F755" t="n">
-        <v>3450</v>
+        <v>4000</v>
       </c>
       <c r="G755" t="inlineStr">
         <is>
@@ -46854,7 +46858,7 @@
       </c>
       <c r="H755" t="inlineStr">
         <is>
-          <t>DeAgostini</t>
+          <t>Altaya</t>
         </is>
       </c>
       <c r="I755" t="inlineStr">
@@ -46875,7 +46879,7 @@
       </c>
       <c r="M755" t="inlineStr">
         <is>
-          <t>MERCEDES-BENZ 300 SLR Racing Sports Car (1955), Mercedes-Benz Offizielle Modell-Sammlung 32, silver</t>
+          <t>Mercedes-Benz 300SLR #722 победитель Mille Miglia 1955 Stilring Moss/Denis Jenkinson (средняя скорость 160км/ч)</t>
         </is>
       </c>
       <c r="N755" t="inlineStr">
@@ -46889,34 +46893,34 @@
         <v>755</v>
       </c>
       <c r="B756" t="n">
-        <v>397000</v>
+        <v>173083</v>
       </c>
       <c r="C756" t="inlineStr">
         <is>
-          <t>​VOISIN Biscooter C-31 1957</t>
+          <t>MERCEDES-BENZ 300 SLR Racing Sports Car 1955</t>
         </is>
       </c>
       <c r="D756" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234313_094.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234643_714.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234316_776.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234309_337.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234305_817.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234320_577.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011339-18.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011339-19.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011339-20.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011339-21.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011339-17.jpg</t>
         </is>
       </c>
       <c r="E756" t="inlineStr">
         <is>
-          <t>7769678</t>
+          <t>7710208</t>
         </is>
       </c>
       <c r="F756" t="n">
-        <v>3500</v>
+        <v>3450</v>
       </c>
       <c r="G756" t="inlineStr">
         <is>
-          <t>Voisin</t>
+          <t>Mercedes-Benz</t>
         </is>
       </c>
       <c r="H756" t="inlineStr">
         <is>
-          <t>Altaya</t>
+          <t>DeAgostini</t>
         </is>
       </c>
       <c r="I756" t="inlineStr">
@@ -46929,11 +46933,7 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K756" t="inlineStr">
-        <is>
-          <t>M2672-26</t>
-        </is>
-      </c>
+      <c r="K756" t="inlineStr"/>
       <c r="L756" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -46941,7 +46941,7 @@
       </c>
       <c r="M756" t="inlineStr">
         <is>
-          <t>VOISIN Biscooter C-31 (1957), Micro-Voitures d'Antan 26</t>
+          <t>MERCEDES-BENZ 300 SLR Racing Sports Car (1955), Mercedes-Benz Offizielle Modell-Sammlung 32, silver</t>
         </is>
       </c>
       <c r="N756" t="inlineStr">
@@ -46955,34 +46955,34 @@
         <v>756</v>
       </c>
       <c r="B757" t="n">
-        <v>348585</v>
+        <v>397000</v>
       </c>
       <c r="C757" t="inlineStr">
         <is>
-          <t>OPEL Blitz M0bel-Werke Eiweilar Saar</t>
+          <t>​VOISIN Biscooter C-31 1957</t>
         </is>
       </c>
       <c r="D757" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000706-1.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000706-2.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000707-1.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000706.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000707.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234313_094.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234643_714.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234316_776.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234309_337.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234305_817.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234320_577.jpg</t>
         </is>
       </c>
       <c r="E757" t="inlineStr">
         <is>
-          <t>7820786</t>
+          <t>7769678</t>
         </is>
       </c>
       <c r="F757" t="n">
-        <v>3250</v>
+        <v>3500</v>
       </c>
       <c r="G757" t="inlineStr">
         <is>
-          <t>Opel</t>
+          <t>Voisin</t>
         </is>
       </c>
       <c r="H757" t="inlineStr">
         <is>
-          <t>DeAgostini</t>
+          <t>Altaya</t>
         </is>
       </c>
       <c r="I757" t="inlineStr">
@@ -46990,8 +46990,16 @@
           <t>1:43</t>
         </is>
       </c>
-      <c r="J757" t="inlineStr"/>
-      <c r="K757" t="inlineStr"/>
+      <c r="J757" t="inlineStr">
+        <is>
+          <t>Металл/пластмасса</t>
+        </is>
+      </c>
+      <c r="K757" t="inlineStr">
+        <is>
+          <t>M2672-26</t>
+        </is>
+      </c>
       <c r="L757" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -46999,7 +47007,7 @@
       </c>
       <c r="M757" t="inlineStr">
         <is>
-          <t>OPEL Blitz M0bel-Werke Eiweilar Saar</t>
+          <t>VOISIN Biscooter C-31 (1957), Micro-Voitures d'Antan 26</t>
         </is>
       </c>
       <c r="N757" t="inlineStr">
@@ -47013,30 +47021,34 @@
         <v>757</v>
       </c>
       <c r="B758" t="n">
-        <v>155503</v>
+        <v>348585</v>
       </c>
       <c r="C758" t="inlineStr">
         <is>
-          <t>MERCEDES-BENZ G4 Francisco Franco 1934</t>
+          <t>OPEL Blitz M0bel-Werke Eiweilar Saar</t>
         </is>
       </c>
       <c r="D758" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234827_382.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234817_976.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234831_408.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234915_733.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234846_582.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234908_315.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234837_787.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234821_522.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234904_469.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000706-1.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000706-2.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000707-1.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000706.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000707.jpg</t>
         </is>
       </c>
       <c r="E758" t="inlineStr">
         <is>
-          <t>7884675</t>
+          <t>7820786</t>
         </is>
       </c>
       <c r="F758" t="n">
-        <v>9000</v>
-      </c>
-      <c r="G758" t="inlineStr"/>
+        <v>3250</v>
+      </c>
+      <c r="G758" t="inlineStr">
+        <is>
+          <t>Opel</t>
+        </is>
+      </c>
       <c r="H758" t="inlineStr">
         <is>
-          <t>Minichamps</t>
+          <t>DeAgostini</t>
         </is>
       </c>
       <c r="I758" t="inlineStr">
@@ -47044,16 +47056,8 @@
           <t>1:43</t>
         </is>
       </c>
-      <c r="J758" t="inlineStr">
-        <is>
-          <t>Металл/пластмасса</t>
-        </is>
-      </c>
-      <c r="K758" t="inlineStr">
-        <is>
-          <t>436035600</t>
-        </is>
-      </c>
+      <c r="J758" t="inlineStr"/>
+      <c r="K758" t="inlineStr"/>
       <c r="L758" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -47061,7 +47065,7 @@
       </c>
       <c r="M758" t="inlineStr">
         <is>
-          <t>MERCEDES-BENZ G4 Francisco Franco, Political leader series 11</t>
+          <t>OPEL Blitz M0bel-Werke Eiweilar Saar</t>
         </is>
       </c>
       <c r="N758" t="inlineStr">
@@ -47075,34 +47079,30 @@
         <v>758</v>
       </c>
       <c r="B759" t="n">
-        <v>375117</v>
+        <v>155503</v>
       </c>
       <c r="C759" t="inlineStr">
         <is>
-          <t>MORRIS MINI MINOR Kultowe Auta 162,</t>
+          <t>MERCEDES-BENZ G4 Francisco Franco 1934</t>
         </is>
       </c>
       <c r="D759" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251206_215504_969.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251206_215459_211.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251206_215501_994.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251206_215456_563.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234827_382.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234817_976.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234831_408.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234915_733.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234846_582.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234908_315.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234837_787.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234821_522.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234904_469.jpg</t>
         </is>
       </c>
       <c r="E759" t="inlineStr">
         <is>
-          <t>8101839</t>
+          <t>7884675</t>
         </is>
       </c>
       <c r="F759" t="n">
-        <v>3000</v>
-      </c>
-      <c r="G759" t="inlineStr">
-        <is>
-          <t>Morris</t>
-        </is>
-      </c>
+        <v>9000</v>
+      </c>
+      <c r="G759" t="inlineStr"/>
       <c r="H759" t="inlineStr">
         <is>
-          <t>DeAgostini</t>
+          <t>Minichamps</t>
         </is>
       </c>
       <c r="I759" t="inlineStr">
@@ -47115,7 +47115,11 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K759" t="inlineStr"/>
+      <c r="K759" t="inlineStr">
+        <is>
+          <t>436035600</t>
+        </is>
+      </c>
       <c r="L759" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -47123,7 +47127,7 @@
       </c>
       <c r="M759" t="inlineStr">
         <is>
-          <t>MORRIS MINI MINOR Kultowe Auta 162,</t>
+          <t>MERCEDES-BENZ G4 Francisco Franco, Political leader series 11</t>
         </is>
       </c>
       <c r="N759" t="inlineStr">
@@ -47137,34 +47141,34 @@
         <v>759</v>
       </c>
       <c r="B760" t="n">
-        <v>182349</v>
+        <v>375117</v>
       </c>
       <c r="C760" t="inlineStr">
         <is>
-          <t>АЦУ-10(52) 1978 г.</t>
+          <t>MORRIS MINI MINOR Kultowe Auta 162,</t>
         </is>
       </c>
       <c r="D760" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-07-11-at-002341-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-07-11-at-002602-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-07-11-at-002611-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-07-11-at-002618-(1).jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251206_215504_969.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251206_215459_211.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251206_215501_994.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251206_215456_563.jpg</t>
         </is>
       </c>
       <c r="E760" t="inlineStr">
         <is>
-          <t>8181608</t>
+          <t>8101839</t>
         </is>
       </c>
       <c r="F760" t="n">
-        <v>8900</v>
+        <v>3000</v>
       </c>
       <c r="G760" t="inlineStr">
         <is>
-          <t>ГАЗ</t>
+          <t>Morris</t>
         </is>
       </c>
       <c r="H760" t="inlineStr">
         <is>
-          <t>DiP Models</t>
+          <t>DeAgostini</t>
         </is>
       </c>
       <c r="I760" t="inlineStr">
@@ -47177,11 +47181,7 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K760" t="inlineStr">
-        <is>
-          <t>105232</t>
-        </is>
-      </c>
+      <c r="K760" t="inlineStr"/>
       <c r="L760" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -47189,7 +47189,7 @@
       </c>
       <c r="M760" t="inlineStr">
         <is>
-          <t>Модель хранилась в боксе. Лот выставлен на других площадках, уточняйте наличие.</t>
+          <t>MORRIS MINI MINOR Kultowe Auta 162,</t>
         </is>
       </c>
       <c r="N760" t="inlineStr">
@@ -47203,30 +47203,34 @@
         <v>760</v>
       </c>
       <c r="B761" t="n">
-        <v>464586</v>
+        <v>182349</v>
       </c>
       <c r="C761" t="inlineStr">
         <is>
-          <t>Local Motors Rally Fighter (2012)</t>
+          <t>АЦУ-10(52) 1978 г.</t>
         </is>
       </c>
       <c r="D761" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260224_161948_852-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260224_162003_308.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260224_162011_706.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260224_161824_589-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260224_161848_637-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260226_005311_332-(1).jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-07-11-at-002341-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-07-11-at-002602-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-07-11-at-002611-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-07-11-at-002618-(1).jpg</t>
         </is>
       </c>
       <c r="E761" t="inlineStr">
         <is>
-          <t>8270561</t>
+          <t>8181608</t>
         </is>
       </c>
       <c r="F761" t="n">
-        <v>5500</v>
-      </c>
-      <c r="G761" t="inlineStr"/>
+        <v>8900</v>
+      </c>
+      <c r="G761" t="inlineStr">
+        <is>
+          <t>ГАЗ</t>
+        </is>
+      </c>
       <c r="H761" t="inlineStr">
         <is>
-          <t>Altaya</t>
+          <t>DiP Models</t>
         </is>
       </c>
       <c r="I761" t="inlineStr">
@@ -47241,7 +47245,7 @@
       </c>
       <c r="K761" t="inlineStr">
         <is>
-          <t>M4069-36</t>
+          <t>105232</t>
         </is>
       </c>
       <c r="L761" t="inlineStr">
@@ -47251,7 +47255,7 @@
       </c>
       <c r="M761" t="inlineStr">
         <is>
-          <t>Local Motors Rally Fighter (2012)</t>
+          <t>Модель хранилась в боксе. Лот выставлен на других площадках, уточняйте наличие.</t>
         </is>
       </c>
       <c r="N761" t="inlineStr">
@@ -47265,34 +47269,30 @@
         <v>761</v>
       </c>
       <c r="B762" t="n">
-        <v>154086</v>
+        <v>464586</v>
       </c>
       <c r="C762" t="inlineStr">
         <is>
-          <t>ЗИС (АМО)-2</t>
+          <t>Local Motors Rally Fighter (2012)</t>
         </is>
       </c>
       <c r="D762" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220533_144.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220535_848.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220602_342.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220527_099.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260224_161948_852-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260224_162003_308.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260224_162011_706.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260224_161824_589-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260224_161848_637-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260226_005311_332-(1).jpg</t>
         </is>
       </c>
       <c r="E762" t="inlineStr">
         <is>
-          <t>8294015</t>
+          <t>8270561</t>
         </is>
       </c>
       <c r="F762" t="n">
-        <v>1950</v>
-      </c>
-      <c r="G762" t="inlineStr">
-        <is>
-          <t>ЗиС</t>
-        </is>
-      </c>
+        <v>5500</v>
+      </c>
+      <c r="G762" t="inlineStr"/>
       <c r="H762" t="inlineStr">
         <is>
-          <t>Наш Автопром</t>
+          <t>Altaya</t>
         </is>
       </c>
       <c r="I762" t="inlineStr">
@@ -47305,7 +47305,11 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K762" t="inlineStr"/>
+      <c r="K762" t="inlineStr">
+        <is>
+          <t>M4069-36</t>
+        </is>
+      </c>
       <c r="L762" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -47313,7 +47317,7 @@
       </c>
       <c r="M762" t="inlineStr">
         <is>
-          <t>ЗИС (АМО)-2</t>
+          <t>Local Motors Rally Fighter (2012)</t>
         </is>
       </c>
       <c r="N762" t="inlineStr">
@@ -47327,30 +47331,34 @@
         <v>762</v>
       </c>
       <c r="B763" t="n">
-        <v>348498</v>
+        <v>154086</v>
       </c>
       <c r="C763" t="inlineStr">
         <is>
-          <t>VANWALL VW57 Formula 1  1957</t>
+          <t>ЗИС (АМО)-2</t>
         </is>
       </c>
       <c r="D763" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-05-at-235227-4.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-05-at-235227-3.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-05-at-235228.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220533_144.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220535_848.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220602_342.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220527_099.jpg</t>
         </is>
       </c>
       <c r="E763" t="inlineStr">
         <is>
-          <t>8363179</t>
+          <t>8294015</t>
         </is>
       </c>
       <c r="F763" t="n">
-        <v>2990</v>
-      </c>
-      <c r="G763" t="inlineStr"/>
+        <v>1950</v>
+      </c>
+      <c r="G763" t="inlineStr">
+        <is>
+          <t>ЗиС</t>
+        </is>
+      </c>
       <c r="H763" t="inlineStr">
         <is>
-          <t>Altaya</t>
+          <t>Наш Автопром</t>
         </is>
       </c>
       <c r="I763" t="inlineStr">
@@ -47371,7 +47379,7 @@
       </c>
       <c r="M763" t="inlineStr">
         <is>
-          <t>VANWALL VW57 Formula 1Stiring Moss 1957</t>
+          <t>ЗИС (АМО)-2</t>
         </is>
       </c>
       <c r="N763" t="inlineStr">
@@ -47385,25 +47393,25 @@
         <v>763</v>
       </c>
       <c r="B764" t="n">
-        <v>440388</v>
+        <v>348498</v>
       </c>
       <c r="C764" t="inlineStr">
         <is>
-          <t>​GOGGOMOBIL TL 400 - 1958</t>
+          <t>VANWALL VW57 Formula 1  1957</t>
         </is>
       </c>
       <c r="D764" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234213_634.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234140_179.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234110_491.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234206_456.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-05-at-235227-4.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-05-at-235227-3.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-05-at-235228.jpg</t>
         </is>
       </c>
       <c r="E764" t="inlineStr">
         <is>
-          <t>846277</t>
+          <t>8363179</t>
         </is>
       </c>
       <c r="F764" t="n">
-        <v>3600</v>
+        <v>2990</v>
       </c>
       <c r="G764" t="inlineStr"/>
       <c r="H764" t="inlineStr">
@@ -47421,11 +47429,7 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K764" t="inlineStr">
-        <is>
-          <t>M2672-44</t>
-        </is>
-      </c>
+      <c r="K764" t="inlineStr"/>
       <c r="L764" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -47433,7 +47437,7 @@
       </c>
       <c r="M764" t="inlineStr">
         <is>
-          <t>GOGGOMOBIL TL 400 - 1958, Micro-Voitures d'Antan 44</t>
+          <t>VANWALL VW57 Formula 1Stiring Moss 1957</t>
         </is>
       </c>
       <c r="N764" t="inlineStr">
@@ -47447,34 +47451,30 @@
         <v>764</v>
       </c>
       <c r="B765" t="n">
-        <v>254037</v>
+        <v>440388</v>
       </c>
       <c r="C765" t="inlineStr">
         <is>
-          <t>​JEEP CJ-7 Renegade 4х4 1983</t>
+          <t>​GOGGOMOBIL TL 400 - 1958</t>
         </is>
       </c>
       <c r="D765" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000407_167.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000405_387.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000341_393.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000326_109.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000407_167-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000412_689-(1).jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234213_634.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234140_179.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234110_491.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234206_456.jpg</t>
         </is>
       </c>
       <c r="E765" t="inlineStr">
         <is>
-          <t>8491610</t>
+          <t>846277</t>
         </is>
       </c>
       <c r="F765" t="n">
-        <v>4600</v>
-      </c>
-      <c r="G765" t="inlineStr">
-        <is>
-          <t>Jeep</t>
-        </is>
-      </c>
+        <v>3600</v>
+      </c>
+      <c r="G765" t="inlineStr"/>
       <c r="H765" t="inlineStr">
         <is>
-          <t>Greenlight Collectibles</t>
+          <t>Altaya</t>
         </is>
       </c>
       <c r="I765" t="inlineStr">
@@ -47489,7 +47489,7 @@
       </c>
       <c r="K765" t="inlineStr">
         <is>
-          <t>86533</t>
+          <t>M2672-44</t>
         </is>
       </c>
       <c r="L765" t="inlineStr">
@@ -47499,7 +47499,7 @@
       </c>
       <c r="M765" t="inlineStr">
         <is>
-          <t>JEEP CJ-7 Renegade 4х4 1983 (машина Сары Коннор из к/ф "Терминатор")</t>
+          <t>GOGGOMOBIL TL 400 - 1958, Micro-Voitures d'Antan 44</t>
         </is>
       </c>
       <c r="N765" t="inlineStr">
@@ -47513,34 +47513,34 @@
         <v>765</v>
       </c>
       <c r="B766" t="n">
-        <v>189066</v>
+        <v>254037</v>
       </c>
       <c r="C766" t="inlineStr">
         <is>
-          <t>PORSCHE 934 #91 24h Le Mans 1980</t>
+          <t>​JEEP CJ-7 Renegade 4х4 1983</t>
         </is>
       </c>
       <c r="D766" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011336-3.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011336-4.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011336-5.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011337.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011336-2.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011337-1.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000407_167.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000405_387.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000341_393.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000326_109.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000407_167-(1).jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251224_000412_689-(1).jpg</t>
         </is>
       </c>
       <c r="E766" t="inlineStr">
         <is>
-          <t>8590544</t>
+          <t>8491610</t>
         </is>
       </c>
       <c r="F766" t="n">
-        <v>7800</v>
+        <v>4600</v>
       </c>
       <c r="G766" t="inlineStr">
         <is>
-          <t>Porsche</t>
+          <t>Jeep</t>
         </is>
       </c>
       <c r="H766" t="inlineStr">
         <is>
-          <t>Premium X</t>
+          <t>Greenlight Collectibles</t>
         </is>
       </c>
       <c r="I766" t="inlineStr">
@@ -47555,7 +47555,7 @@
       </c>
       <c r="K766" t="inlineStr">
         <is>
-          <t>PR0417</t>
+          <t>86533</t>
         </is>
       </c>
       <c r="L766" t="inlineStr">
@@ -47565,7 +47565,7 @@
       </c>
       <c r="M766" t="inlineStr">
         <is>
-          <t>PORSCHE 934 #91 24h Le Mans 1980есть другие</t>
+          <t>JEEP CJ-7 Renegade 4х4 1983 (машина Сары Коннор из к/ф "Терминатор")</t>
         </is>
       </c>
       <c r="N766" t="inlineStr">
@@ -47579,34 +47579,34 @@
         <v>766</v>
       </c>
       <c r="B767" t="n">
-        <v>396798</v>
+        <v>189066</v>
       </c>
       <c r="C767" t="inlineStr">
         <is>
-          <t>MERCEDES-BENZ 500 SEL W126  1989</t>
+          <t>PORSCHE 934 #91 24h Le Mans 1980</t>
         </is>
       </c>
       <c r="D767" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251231_000901_934.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251231_000858_102.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251231_000852_805.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251231_000730_668.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251231_000853_965.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251231_000900_979.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011336-3.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011336-4.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011336-5.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011337.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011336-2.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011337-1.jpg</t>
         </is>
       </c>
       <c r="E767" t="inlineStr">
         <is>
-          <t>8614264</t>
+          <t>8590544</t>
         </is>
       </c>
       <c r="F767" t="n">
-        <v>9800</v>
+        <v>7800</v>
       </c>
       <c r="G767" t="inlineStr">
         <is>
-          <t>Mercedes-Benz</t>
+          <t>Porsche</t>
         </is>
       </c>
       <c r="H767" t="inlineStr">
         <is>
-          <t>Minichamps</t>
+          <t>Premium X</t>
         </is>
       </c>
       <c r="I767" t="inlineStr">
@@ -47619,7 +47619,11 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K767" t="inlineStr"/>
+      <c r="K767" t="inlineStr">
+        <is>
+          <t>PR0417</t>
+        </is>
+      </c>
       <c r="L767" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -47627,7 +47631,7 @@
       </c>
       <c r="M767" t="inlineStr">
         <is>
-          <t>MERCEDES-BENZ 500 SEL W126 Helmut Kohl (1989), silver</t>
+          <t>PORSCHE 934 #91 24h Le Mans 1980есть другие</t>
         </is>
       </c>
       <c r="N767" t="inlineStr">
@@ -47641,30 +47645,34 @@
         <v>767</v>
       </c>
       <c r="B768" t="n">
-        <v>397723</v>
+        <v>396798</v>
       </c>
       <c r="C768" t="inlineStr">
         <is>
-          <t>Rovin D4 1963</t>
+          <t>MERCEDES-BENZ 500 SEL W126  1989</t>
         </is>
       </c>
       <c r="D768" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234250_715.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234254_169.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234258_169.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234301_635.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251231_000901_934.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251231_000858_102.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251231_000852_805.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251231_000730_668.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251231_000853_965.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251231_000900_979.jpg</t>
         </is>
       </c>
       <c r="E768" t="inlineStr">
         <is>
-          <t>8730208</t>
+          <t>8614264</t>
         </is>
       </c>
       <c r="F768" t="n">
-        <v>3400</v>
-      </c>
-      <c r="G768" t="inlineStr"/>
+        <v>9800</v>
+      </c>
+      <c r="G768" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
       <c r="H768" t="inlineStr">
         <is>
-          <t>Altaya</t>
+          <t>Minichamps</t>
         </is>
       </c>
       <c r="I768" t="inlineStr">
@@ -47677,11 +47685,7 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K768" t="inlineStr">
-        <is>
-          <t>M2672-04</t>
-        </is>
-      </c>
+      <c r="K768" t="inlineStr"/>
       <c r="L768" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -47689,7 +47693,7 @@
       </c>
       <c r="M768" t="inlineStr">
         <is>
-          <t>Rovin D4 1954, Micro-Voitures d'Antan 4</t>
+          <t>MERCEDES-BENZ 500 SEL W126 Helmut Kohl (1989), silver</t>
         </is>
       </c>
       <c r="N768" t="inlineStr">
@@ -47703,31 +47707,27 @@
         <v>768</v>
       </c>
       <c r="B769" t="n">
-        <v>181009</v>
+        <v>397723</v>
       </c>
       <c r="C769" t="inlineStr">
         <is>
-          <t>MERCEDES-BENZ 240 D Long 1973</t>
+          <t>Rovin D4 1963</t>
         </is>
       </c>
       <c r="D769" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-20.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-21.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-22.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-19.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234250_715.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234254_169.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234258_169.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234301_635.jpg</t>
         </is>
       </c>
       <c r="E769" t="inlineStr">
         <is>
-          <t>8764360</t>
+          <t>8730208</t>
         </is>
       </c>
       <c r="F769" t="n">
-        <v>4800</v>
-      </c>
-      <c r="G769" t="inlineStr">
-        <is>
-          <t>Mercedes-Benz</t>
-        </is>
-      </c>
+        <v>3400</v>
+      </c>
+      <c r="G769" t="inlineStr"/>
       <c r="H769" t="inlineStr">
         <is>
           <t>Altaya</t>
@@ -47743,7 +47743,11 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K769" t="inlineStr"/>
+      <c r="K769" t="inlineStr">
+        <is>
+          <t>M2672-04</t>
+        </is>
+      </c>
       <c r="L769" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -47751,7 +47755,7 @@
       </c>
       <c r="M769" t="inlineStr">
         <is>
-          <t>MERCEDES-BENZ 240 D Long (1973)</t>
+          <t>Rovin D4 1954, Micro-Voitures d'Antan 4</t>
         </is>
       </c>
       <c r="N769" t="inlineStr">
@@ -47765,29 +47769,29 @@
         <v>769</v>
       </c>
       <c r="B770" t="n">
-        <v>197683</v>
+        <v>181009</v>
       </c>
       <c r="C770" t="inlineStr">
         <is>
-          <t>MASERATI Tipo 61 #78 1961</t>
+          <t>MERCEDES-BENZ 240 D Long 1973</t>
         </is>
       </c>
       <c r="D770" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230055.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230056.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230054.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230057.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230055-1.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-20.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-21.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-22.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-29-at-011338-19.jpg</t>
         </is>
       </c>
       <c r="E770" t="inlineStr">
         <is>
-          <t>8805103</t>
+          <t>8764360</t>
         </is>
       </c>
       <c r="F770" t="n">
-        <v>3500</v>
+        <v>4800</v>
       </c>
       <c r="G770" t="inlineStr">
         <is>
-          <t>Maserati</t>
+          <t>Mercedes-Benz</t>
         </is>
       </c>
       <c r="H770" t="inlineStr">
@@ -47805,11 +47809,7 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K770" t="inlineStr">
-        <is>
-          <t>MA062</t>
-        </is>
-      </c>
+      <c r="K770" t="inlineStr"/>
       <c r="L770" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -47817,7 +47817,7 @@
       </c>
       <c r="M770" t="inlineStr">
         <is>
-          <t>MASERATI Tipo 61 #78 Schroeder Nassau Trophy 1961</t>
+          <t>MERCEDES-BENZ 240 D Long (1973)</t>
         </is>
       </c>
       <c r="N770" t="inlineStr">
@@ -47831,29 +47831,29 @@
         <v>770</v>
       </c>
       <c r="B771" t="n">
-        <v>185683</v>
+        <v>197683</v>
       </c>
       <c r="C771" t="inlineStr">
         <is>
-          <t>Seat Cordoba WRC #2 (2001)</t>
+          <t>MASERATI Tipo 61 #78 1961</t>
         </is>
       </c>
       <c r="D771" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-13-at-022720-1.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-13-at-022720-4.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-13-at-022720-3.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230055.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230056.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230054.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230057.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-11-03-at-230055-1.jpg</t>
         </is>
       </c>
       <c r="E771" t="inlineStr">
         <is>
-          <t>896156</t>
+          <t>8805103</t>
         </is>
       </c>
       <c r="F771" t="n">
-        <v>3800</v>
+        <v>3500</v>
       </c>
       <c r="G771" t="inlineStr">
         <is>
-          <t>SEAT</t>
+          <t>Maserati</t>
         </is>
       </c>
       <c r="H771" t="inlineStr">
@@ -47871,7 +47871,11 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K771" t="inlineStr"/>
+      <c r="K771" t="inlineStr">
+        <is>
+          <t>MA062</t>
+        </is>
+      </c>
       <c r="L771" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -47879,7 +47883,7 @@
       </c>
       <c r="M771" t="inlineStr">
         <is>
-          <t>Seat Cordoba WRC #2 Rally RAC Navarra de Tierra, 2001</t>
+          <t>MASERATI Tipo 61 #78 Schroeder Nassau Trophy 1961</t>
         </is>
       </c>
       <c r="N771" t="inlineStr">
@@ -47893,29 +47897,29 @@
         <v>771</v>
       </c>
       <c r="B772" t="n">
-        <v>225471</v>
+        <v>185683</v>
       </c>
       <c r="C772" t="inlineStr">
         <is>
-          <t>LAMBORGHINI Diablo VT-R Roadster Trofeo 1997</t>
+          <t>Seat Cordoba WRC #2 (2001)</t>
         </is>
       </c>
       <c r="D772" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234324_300.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234640_247.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234634_264.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234638_048.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234631_600.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234625_500.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234641_985.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234627_491.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-13-at-022720-1.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-13-at-022720-4.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-13-at-022720-3.jpg</t>
         </is>
       </c>
       <c r="E772" t="inlineStr">
         <is>
-          <t>9017121</t>
+          <t>896156</t>
         </is>
       </c>
       <c r="F772" t="n">
-        <v>4000</v>
+        <v>3800</v>
       </c>
       <c r="G772" t="inlineStr">
         <is>
-          <t>Lamborghini</t>
+          <t>SEAT</t>
         </is>
       </c>
       <c r="H772" t="inlineStr">
@@ -47933,11 +47937,7 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K772" t="inlineStr">
-        <is>
-          <t>LAM052</t>
-        </is>
-      </c>
+      <c r="K772" t="inlineStr"/>
       <c r="L772" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -47945,7 +47945,7 @@
       </c>
       <c r="M772" t="inlineStr">
         <is>
-          <t>LAMBORGHINI Diablo VT-R Roadster Trofeo 1997</t>
+          <t>Seat Cordoba WRC #2 Rally RAC Navarra de Tierra, 2001</t>
         </is>
       </c>
       <c r="N772" t="inlineStr">
@@ -47959,27 +47959,31 @@
         <v>772</v>
       </c>
       <c r="B773" t="n">
-        <v>317708</v>
+        <v>225471</v>
       </c>
       <c r="C773" t="inlineStr">
         <is>
-          <t>FIAT 125 Mirafiori 1981</t>
+          <t>LAMBORGHINI Diablo VT-R Roadster Trofeo 1997</t>
         </is>
       </c>
       <c r="D773" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220203_741.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220307_178.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220126_625.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220430_080.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220342_780.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220330_259.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220252_274.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234324_300.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234640_247.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234634_264.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234638_048.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234631_600.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234625_500.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234641_985.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20251208_234627_491.jpg</t>
         </is>
       </c>
       <c r="E773" t="inlineStr">
         <is>
-          <t>9127780</t>
+          <t>9017121</t>
         </is>
       </c>
       <c r="F773" t="n">
-        <v>2300</v>
-      </c>
-      <c r="G773" t="inlineStr"/>
+        <v>4000</v>
+      </c>
+      <c r="G773" t="inlineStr">
+        <is>
+          <t>Lamborghini</t>
+        </is>
+      </c>
       <c r="H773" t="inlineStr">
         <is>
           <t>Altaya</t>
@@ -47995,7 +47999,11 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K773" t="inlineStr"/>
+      <c r="K773" t="inlineStr">
+        <is>
+          <t>LAM052</t>
+        </is>
+      </c>
       <c r="L773" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -48003,7 +48011,7 @@
       </c>
       <c r="M773" t="inlineStr">
         <is>
-          <t>FIAT 125 Mirafiori (1981)надломано переднее левое колесо</t>
+          <t>LAMBORGHINI Diablo VT-R Roadster Trofeo 1997</t>
         </is>
       </c>
       <c r="N773" t="inlineStr">
@@ -48017,31 +48025,27 @@
         <v>773</v>
       </c>
       <c r="B774" t="n">
-        <v>257979</v>
+        <v>317708</v>
       </c>
       <c r="C774" t="inlineStr">
         <is>
-          <t>Seat Ibiza GTI Kit Car #24 (1999)</t>
+          <t>FIAT 125 Mirafiori 1981</t>
         </is>
       </c>
       <c r="D774" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221300-7.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221300-8.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221300-9.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220203_741.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220307_178.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220126_625.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220430_080.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220342_780.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220330_259.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260526_220252_274.jpg</t>
         </is>
       </c>
       <c r="E774" t="inlineStr">
         <is>
-          <t>9131472</t>
+          <t>9127780</t>
         </is>
       </c>
       <c r="F774" t="n">
-        <v>4200</v>
-      </c>
-      <c r="G774" t="inlineStr">
-        <is>
-          <t>SEAT</t>
-        </is>
-      </c>
+        <v>2300</v>
+      </c>
+      <c r="G774" t="inlineStr"/>
       <c r="H774" t="inlineStr">
         <is>
           <t>Altaya</t>
@@ -48065,7 +48069,7 @@
       </c>
       <c r="M774" t="inlineStr">
         <is>
-          <t>Seat Ibiza GTI Kit Car #24 Rally Monte-Carlo (1999)</t>
+          <t>FIAT 125 Mirafiori (1981)надломано переднее левое колесо</t>
         </is>
       </c>
       <c r="N774" t="inlineStr">
@@ -48079,34 +48083,34 @@
         <v>774</v>
       </c>
       <c r="B775" t="n">
-        <v>176461</v>
+        <v>257979</v>
       </c>
       <c r="C775" t="inlineStr">
         <is>
-          <t>Уральский 375Д бортовой с тентом</t>
+          <t>Seat Ibiza GTI Kit Car #24 (1999)</t>
         </is>
       </c>
       <c r="D775" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-10-29-at-234457-5.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-10-29-at-234457-7.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-10-29-at-234457-4.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-07-08-at-233410-(1).jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221300-7.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221300-8.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-12-at-221300-9.jpg</t>
         </is>
       </c>
       <c r="E775" t="inlineStr">
         <is>
-          <t>9192234</t>
+          <t>9131472</t>
         </is>
       </c>
       <c r="F775" t="n">
-        <v>4350</v>
+        <v>4200</v>
       </c>
       <c r="G775" t="inlineStr">
         <is>
-          <t>УРАЛ</t>
+          <t>SEAT</t>
         </is>
       </c>
       <c r="H775" t="inlineStr">
         <is>
-          <t>Start Scale Models (SSM)</t>
+          <t>Altaya</t>
         </is>
       </c>
       <c r="I775" t="inlineStr">
@@ -48119,11 +48123,7 @@
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K775" t="inlineStr">
-        <is>
-          <t>SSM1103</t>
-        </is>
-      </c>
+      <c r="K775" t="inlineStr"/>
       <c r="L775" t="inlineStr">
         <is>
           <t>Новый</t>
@@ -48131,7 +48131,7 @@
       </c>
       <c r="M775" t="inlineStr">
         <is>
-          <t>Уральский 375Д бортовой с тентом, голубой</t>
+          <t>Seat Ibiza GTI Kit Car #24 Rally Monte-Carlo (1999)</t>
         </is>
       </c>
       <c r="N775" t="inlineStr">
@@ -48145,34 +48145,34 @@
         <v>775</v>
       </c>
       <c r="B776" t="n">
-        <v>189538</v>
+        <v>176461</v>
       </c>
       <c r="C776" t="inlineStr">
         <is>
-          <t>Mersedes-Benz CLS 350</t>
+          <t>Уральский 375Д бортовой с тентом</t>
         </is>
       </c>
       <c r="D776" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-15.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-19.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-16.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-17.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-14.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-18.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-10-29-at-234457-5.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-10-29-at-234457-7.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-10-29-at-234457-4.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-07-08-at-233410-(1).jpg</t>
         </is>
       </c>
       <c r="E776" t="inlineStr">
         <is>
-          <t>9579352</t>
+          <t>9192234</t>
         </is>
       </c>
       <c r="F776" t="n">
-        <v>5600</v>
+        <v>4350</v>
       </c>
       <c r="G776" t="inlineStr">
         <is>
-          <t>Mercedes-Benz</t>
+          <t>УРАЛ</t>
         </is>
       </c>
       <c r="H776" t="inlineStr">
         <is>
-          <t>Norev</t>
+          <t>Start Scale Models (SSM)</t>
         </is>
       </c>
       <c r="I776" t="inlineStr">
@@ -48187,7 +48187,7 @@
       </c>
       <c r="K776" t="inlineStr">
         <is>
-          <t>400020101</t>
+          <t>SSM1103</t>
         </is>
       </c>
       <c r="L776" t="inlineStr">
@@ -48197,7 +48197,7 @@
       </c>
       <c r="M776" t="inlineStr">
         <is>
-          <t>Mersedes-Benz CLS 350 от Norel</t>
+          <t>Уральский 375Д бортовой с тентом, голубой</t>
         </is>
       </c>
       <c r="N776" t="inlineStr">
@@ -48211,34 +48211,34 @@
         <v>776</v>
       </c>
       <c r="B777" t="n">
-        <v>174204</v>
+        <v>189538</v>
       </c>
       <c r="C777" t="inlineStr">
         <is>
-          <t>RANGE ROVER Sport Casino Royale (2006)</t>
+          <t>Mersedes-Benz CLS 350</t>
         </is>
       </c>
       <c r="D777" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012216-23.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012216-24.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012216-25.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-15.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-19.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-16.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-17.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-14.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-04-at-000223-18.jpg</t>
         </is>
       </c>
       <c r="E777" t="inlineStr">
         <is>
-          <t>9661295</t>
+          <t>9579352</t>
         </is>
       </c>
       <c r="F777" t="n">
-        <v>3500</v>
+        <v>5600</v>
       </c>
       <c r="G777" t="inlineStr">
         <is>
-          <t>Rover</t>
+          <t>Mercedes-Benz</t>
         </is>
       </c>
       <c r="H777" t="inlineStr">
         <is>
-          <t>Eaglemoss</t>
+          <t>Norev</t>
         </is>
       </c>
       <c r="I777" t="inlineStr">
@@ -48253,7 +48253,7 @@
       </c>
       <c r="K777" t="inlineStr">
         <is>
-          <t>JB51</t>
+          <t>400020101</t>
         </is>
       </c>
       <c r="L777" t="inlineStr">
@@ -48263,7 +48263,7 @@
       </c>
       <c r="M777" t="inlineStr">
         <is>
-          <t>RANGE ROVER Sport Casino Royale (2006), metallic gold</t>
+          <t>Mersedes-Benz CLS 350 от Norel</t>
         </is>
       </c>
       <c r="N777" t="inlineStr">
@@ -48277,34 +48277,34 @@
         <v>777</v>
       </c>
       <c r="B778" t="n">
-        <v>155500</v>
+        <v>174204</v>
       </c>
       <c r="C778" t="inlineStr">
         <is>
-          <t>Alfa Romeo 8C 2900 B Lungo 1938</t>
+          <t>RANGE ROVER Sport Casino Royale (2006)</t>
         </is>
       </c>
       <c r="D778" t="inlineStr">
         <is>
-          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_235004_019.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234956_550.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_235011_631.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_235000_296.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234952_900.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_235015_299.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_235032_770.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_235025_966.jpg</t>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012216-23.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012216-24.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012216-25.jpg</t>
         </is>
       </c>
       <c r="E778" t="inlineStr">
         <is>
-          <t>9711764</t>
+          <t>9661295</t>
         </is>
       </c>
       <c r="F778" t="n">
-        <v>9500</v>
+        <v>3500</v>
       </c>
       <c r="G778" t="inlineStr">
         <is>
-          <t>Alfa Romeo</t>
+          <t>Rover</t>
         </is>
       </c>
       <c r="H778" t="inlineStr">
         <is>
-          <t>Minichamps</t>
+          <t>Eaglemoss</t>
         </is>
       </c>
       <c r="I778" t="inlineStr">
@@ -48319,7 +48319,7 @@
       </c>
       <c r="K778" t="inlineStr">
         <is>
-          <t>TSMCE154313</t>
+          <t>JB51</t>
         </is>
       </c>
       <c r="L778" t="inlineStr">
@@ -48329,7 +48329,7 @@
       </c>
       <c r="M778" t="inlineStr">
         <is>
-          <t>Alfa Romeo 8C 2900 B Lungo Touring Carrozzeria Superleggera</t>
+          <t>RANGE ROVER Sport Casino Royale (2006), metallic gold</t>
         </is>
       </c>
       <c r="N778" t="inlineStr">
@@ -48343,62 +48343,194 @@
         <v>778</v>
       </c>
       <c r="B779" t="n">
+        <v>155500</v>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>Alfa Romeo 8C 2900 B Lungo 1938</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_235004_019.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234956_550.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_235011_631.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_235000_296.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_234952_900.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_235015_299.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_235032_770.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/img_20260505_235025_966.jpg</t>
+        </is>
+      </c>
+      <c r="E779" t="inlineStr">
+        <is>
+          <t>9711764</t>
+        </is>
+      </c>
+      <c r="F779" t="n">
+        <v>9500</v>
+      </c>
+      <c r="G779" t="inlineStr">
+        <is>
+          <t>Alfa Romeo</t>
+        </is>
+      </c>
+      <c r="H779" t="inlineStr">
+        <is>
+          <t>Minichamps</t>
+        </is>
+      </c>
+      <c r="I779" t="inlineStr">
+        <is>
+          <t>1:43</t>
+        </is>
+      </c>
+      <c r="J779" t="inlineStr">
+        <is>
+          <t>Металл/пластмасса</t>
+        </is>
+      </c>
+      <c r="K779" t="inlineStr">
+        <is>
+          <t>TSMCE154313</t>
+        </is>
+      </c>
+      <c r="L779" t="inlineStr">
+        <is>
+          <t>Новый</t>
+        </is>
+      </c>
+      <c r="M779" t="inlineStr">
+        <is>
+          <t>Alfa Romeo 8C 2900 B Lungo Touring Carrozzeria Superleggera</t>
+        </is>
+      </c>
+      <c r="N779" t="inlineStr">
+        <is>
+          <t>Россия, Хабаровский край, Хабаровск</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="n">
+        <v>779</v>
+      </c>
+      <c r="B780" t="n">
+        <v>184756</v>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>MITSUBISHI LANCER EVOLUTION X - #61</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012217-1.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012217-4.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012217-3.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012217-2.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-08-12-at-012217.jpg</t>
+        </is>
+      </c>
+      <c r="E780" t="inlineStr">
+        <is>
+          <t>9864273</t>
+        </is>
+      </c>
+      <c r="F780" t="n">
+        <v>6100</v>
+      </c>
+      <c r="G780" t="inlineStr">
+        <is>
+          <t>Mitsubishi</t>
+        </is>
+      </c>
+      <c r="H780" t="inlineStr">
+        <is>
+          <t>Vitesse</t>
+        </is>
+      </c>
+      <c r="I780" t="inlineStr">
+        <is>
+          <t>1:43</t>
+        </is>
+      </c>
+      <c r="J780" t="inlineStr">
+        <is>
+          <t>Металл/пластмасса</t>
+        </is>
+      </c>
+      <c r="K780" t="inlineStr">
+        <is>
+          <t>43428</t>
+        </is>
+      </c>
+      <c r="L780" t="inlineStr">
+        <is>
+          <t>Новый</t>
+        </is>
+      </c>
+      <c r="M780" t="inlineStr">
+        <is>
+          <t>MITSUBISHI LANCER EVOLUTION X - #61 F.Nutahara/T.Sato</t>
+        </is>
+      </c>
+      <c r="N780" t="inlineStr">
+        <is>
+          <t>Россия, Хабаровский край, Хабаровск</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="n">
+        <v>780</v>
+      </c>
+      <c r="B781" t="n">
         <v>8091</v>
       </c>
-      <c r="C779" t="inlineStr">
+      <c r="C781" t="inlineStr">
         <is>
           <t>ROCAR TV 12F</t>
         </is>
       </c>
-      <c r="D779" t="inlineStr">
+      <c r="D781" t="inlineStr">
         <is>
           <t>https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-08-at-012435-1.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-08-at-012435-2.jpg; https://scalebay.ru/uploads/user/s/a/sanya-kuznec_7522/whatsapp-image-2025-09-08-at-012436.jpg</t>
         </is>
       </c>
-      <c r="E779" t="inlineStr">
+      <c r="E781" t="inlineStr">
         <is>
           <t>9896814</t>
         </is>
       </c>
-      <c r="F779" t="n">
+      <c r="F781" t="n">
         <v>2050</v>
       </c>
-      <c r="G779" t="inlineStr">
+      <c r="G781" t="inlineStr">
         <is>
           <t>Rocar</t>
         </is>
       </c>
-      <c r="H779" t="inlineStr">
+      <c r="H781" t="inlineStr">
         <is>
           <t>DeAgostini</t>
         </is>
       </c>
-      <c r="I779" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="J779" t="inlineStr">
+      <c r="I781" t="inlineStr">
+        <is>
+          <t>1:43</t>
+        </is>
+      </c>
+      <c r="J781" t="inlineStr">
         <is>
           <t>Металл/пластмасса</t>
         </is>
       </c>
-      <c r="K779" t="inlineStr">
+      <c r="K781" t="inlineStr">
         <is>
           <t>mas017</t>
         </is>
       </c>
-      <c r="L779" t="inlineStr">
-        <is>
-          <t>Новый</t>
-        </is>
-      </c>
-      <c r="M779" t="inlineStr">
+      <c r="L781" t="inlineStr">
+        <is>
+          <t>Новый</t>
+        </is>
+      </c>
+      <c r="M781" t="inlineStr">
         <is>
           <t>ROCAR TV 12F, Masini de Legenda 17, yellow№ 17 из серии Мașini de legendă</t>
         </is>
       </c>
-      <c r="N779" t="inlineStr">
+      <c r="N781" t="inlineStr">
         <is>
           <t>Россия, Хабаровский край, Хабаровск</t>
         </is>

</xml_diff>

<commit_message>
Update matched_far.xlsx (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -413,298 +413,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>№</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>ID UNOMAG</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Название</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Фото (ссылки)</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Лот №</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Единая цена</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Марка</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Производитель</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Масштаб</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Материал</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Артикул</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Состояние</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Описание</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Местоположение</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="n">
-        <v>226818</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mercedes Brabus 850 6.0 Widestar  2016 Minichamps</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20260202_134535.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20260202_134448.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20260202_134541.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20260202_134547.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20260202_134601.jpg</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>4213802</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>9500</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Mercedes-Benz</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Minichamps</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Б/у</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>В связи с колебаниями курса рубля, необходимо уточнять цену перед покупкой.Отправляю по всему миру - по возможности.</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="n">
-        <v>176749</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Mercedes Brabus G  V12 Widestar 2010  Minichamps</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175143.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175106.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175136.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175148.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/img_20251028_175203.jpg</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>7151583</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>9500</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Brabus</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Minichamps</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Б/у</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>В связи с колебаниями курса рубля, необходимо уточнять цену перед покупкой.Отправляю по всему миру - по возможности.</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>214388</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Audi RS4 RS 4 Avant  2018 Spark</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471219.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471242.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471236.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471229.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471223.jpg; https://scalebay.ru/uploads/user/f/o/fortythird_3839/1712674471213.jpg</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>9331546</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>9600</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Audi</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Spark</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Новый</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>В связи с колебаниями курса рубля, необходимо уточнять цену перед покупкой.Привезу любые модели на заказ.</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="n">
-        <v>484586</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Skoda 706 RTTN с полуприцепом Alka N12CH   АИСТ</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-2.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-3.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-8.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-9.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-6.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-7.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-5.jpg; https://scalebay.ru/uploads/user/l/a/labtoz_20/skoda-706-rttn-s-polupricepom-alka-n12ch-114510-10.jpg</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>7409184</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>4100</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Škoda</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Автоистория (АИСТ)</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>1:43</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>металл , пластик, резина</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Новый</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Информация по оплате и отправке в разделе " Обо мне". Условия аукциона стандартные. выход на связь в течении 3 дней оплата в течении 7 дней с момента окончания аукциона. Все вопросы по лоту , оплате , отправке исключительно до покупки (до ставки) Смотрите мои другие лоты.</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update matched_far.xlsx (2 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -413,9 +413,198 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>234689</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Mercedes X-Class 2017</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/user/m/a/mandiby_7644/mercedes-x-klasse-norev-183421-6.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20200121_202209.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20200121_202532.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20200121_202227.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20200121_202414.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20200121_202238.jpg; https://scalebay.ru/uploads/user/m/a/mandiby_7644/20200121_202319.jpg</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>4439325</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>9598</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Norev</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>1:18</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Новый</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Модель абсолютно новая.доставалась из коробки только для фотографирования.При отправке почтой,гарантирую надежную упаковку.Возможно объединение нескольких лотов. Отвечу на все Ваши вопросы (до покупки)</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>652272</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>КамАЗ-6522 самосвал белый</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://scalebay.ru/uploads/user/a/v/avtobusnik_6320/kamaz-6522-655359-2.jpg; https://scalebay.ru/uploads/user/a/v/avtobusnik_6320/kamaz-6522-655359-1.jpg; https://scalebay.ru/uploads/user/a/v/avtobusnik_6320/kamaz-6522-655359-4.jpg; https://scalebay.ru/uploads/user/a/v/avtobusnik_6320/kamaz-6522-655359-3.jpg; https://scalebay.ru/uploads/user/a/v/avtobusnik_6320/kamaz-6522-655359-7.jpg; https://scalebay.ru/uploads/user/a/v/avtobusnik_6320/kamaz-6522-655359-5.jpg; https://scalebay.ru/uploads/user/a/v/avtobusnik_6320/kamaz-6522-655359-8.jpg</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1613562</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>4200</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>КамАЗ</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>ПАО КАМАЗ</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>1:43</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Металл/пластмасса</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>104165</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Новый</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Модель новая в оригинальной упаковке.Самовывоз в Москве от метро Строгино.Почта России или СДЭК от 500 рублей.Выход на связь 1 день, оплата на карту Альфа банка 5 дней.</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-08-21 05:44 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-08-21 06:15 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
scalebay update 2026-09-01 03:04 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-04 05:36 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-04 18:03 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-05 06:28 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-05 18:49 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-06 07:12 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-07 08:01 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-08 21:14 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-09 09:39 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-09 22:07 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-10 10:31 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-10 23:05 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-11 11:33 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-12 00:05 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
scalebay update 2026-09-13 00:59 (0 lots)
</commit_message>
<xml_diff>
--- a/matched_far.xlsx
+++ b/matched_far.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matched Far" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +433,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ID UNOMAG</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Название</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Фото (ссылки)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Лот №</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Единая цена</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Марка</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Производитель</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Масштаб</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Артикул</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Состояние</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Описание</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Наличие</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>